<commit_message>
[fix] modification du powerpoint
</commit_message>
<xml_diff>
--- a/cv/AYAD_Ademe_TableauSynthese.xlsx
+++ b/cv/AYAD_Ademe_TableauSynthese.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\boulo\Desktop\E5\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp64\www\AYAD\AYAD_Ademe_Portfolio\cv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDF35319-7654-46E7-925C-AEC8005F13DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFD86C93-C32C-4316-9A00-85643183DB35}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="29020" windowHeight="15700" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="51">
   <si>
     <t>BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
@@ -205,6 +205,12 @@
   </si>
   <si>
     <t>N° candidat : 101047555GB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Projet HSP Symfony </t>
+  </si>
+  <si>
+    <t>09/09/2025 au 09/12/2025</t>
   </si>
 </sst>
 </file>
@@ -741,9 +747,48 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -766,45 +811,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1126,56 +1132,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
-      <c r="G1" s="22" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24" t="s">
         <v>47</v>
       </c>
-      <c r="H1" s="22"/>
+      <c r="H1" s="24"/>
     </row>
     <row r="2" spans="1:43" ht="41.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="22"/>
-      <c r="C2" s="22"/>
-      <c r="D2" s="22"/>
-      <c r="E2" s="22"/>
-      <c r="F2" s="22"/>
-      <c r="G2" s="22"/>
-      <c r="H2" s="22"/>
+      <c r="B2" s="24"/>
+      <c r="C2" s="24"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="24"/>
+      <c r="H2" s="24"/>
     </row>
     <row r="3" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="25"/>
-      <c r="F3" s="29" t="s">
+      <c r="B3" s="37"/>
+      <c r="C3" s="37"/>
+      <c r="D3" s="37"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="42" t="s">
         <v>48</v>
       </c>
-      <c r="G3" s="24"/>
-      <c r="H3" s="30"/>
+      <c r="G3" s="37"/>
+      <c r="H3" s="43"/>
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:43" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="26" t="s">
+      <c r="A4" s="39" t="s">
         <v>42</v>
       </c>
-      <c r="B4" s="27"/>
-      <c r="C4" s="27"/>
-      <c r="D4" s="27"/>
-      <c r="E4" s="28"/>
+      <c r="B4" s="40"/>
+      <c r="C4" s="40"/>
+      <c r="D4" s="40"/>
+      <c r="E4" s="41"/>
       <c r="F4" s="12" t="s">
         <v>2</v>
       </c>
@@ -1187,22 +1193,22 @@
       </c>
     </row>
     <row r="5" spans="1:43" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="41" t="s">
+      <c r="A5" s="33" t="s">
         <v>46</v>
       </c>
-      <c r="B5" s="42"/>
-      <c r="C5" s="42"/>
-      <c r="D5" s="42"/>
-      <c r="E5" s="42"/>
-      <c r="F5" s="42"/>
-      <c r="G5" s="42"/>
-      <c r="H5" s="43"/>
+      <c r="B5" s="34"/>
+      <c r="C5" s="34"/>
+      <c r="D5" s="34"/>
+      <c r="E5" s="34"/>
+      <c r="F5" s="34"/>
+      <c r="G5" s="34"/>
+      <c r="H5" s="35"/>
     </row>
     <row r="6" spans="1:43" ht="90" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="31" t="s">
+      <c r="A6" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="39" t="s">
+      <c r="B6" s="31" t="s">
         <v>5</v>
       </c>
       <c r="C6" s="6" t="s">
@@ -1225,8 +1231,8 @@
       </c>
     </row>
     <row r="7" spans="1:43" s="2" customFormat="1" ht="325" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="32"/>
-      <c r="B7" s="40"/>
+      <c r="A7" s="23"/>
+      <c r="B7" s="32"/>
       <c r="C7" s="19" t="s">
         <v>12</v>
       </c>
@@ -1282,16 +1288,16 @@
       <c r="AQ7"/>
     </row>
     <row r="8" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A8" s="33" t="s">
+      <c r="A8" s="25" t="s">
         <v>18</v>
       </c>
-      <c r="B8" s="34"/>
-      <c r="C8" s="34"/>
-      <c r="D8" s="34"/>
-      <c r="E8" s="34"/>
-      <c r="F8" s="34"/>
-      <c r="G8" s="34"/>
-      <c r="H8" s="35"/>
+      <c r="B8" s="26"/>
+      <c r="C8" s="26"/>
+      <c r="D8" s="26"/>
+      <c r="E8" s="26"/>
+      <c r="F8" s="26"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="27"/>
       <c r="I8"/>
       <c r="J8"/>
       <c r="K8"/>
@@ -1695,8 +1701,12 @@
       <c r="AQ15"/>
     </row>
     <row r="16" spans="1:43" s="2" customFormat="1" ht="40" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="9"/>
-      <c r="B16" s="8"/>
+      <c r="A16" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B16" s="8" t="s">
+        <v>50</v>
+      </c>
       <c r="C16" s="14"/>
       <c r="D16" s="14"/>
       <c r="E16" s="14"/>
@@ -1830,16 +1840,16 @@
       <c r="AQ18"/>
     </row>
     <row r="19" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A19" s="36" t="s">
+      <c r="A19" s="28" t="s">
         <v>19</v>
       </c>
-      <c r="B19" s="37"/>
-      <c r="C19" s="37"/>
-      <c r="D19" s="37"/>
-      <c r="E19" s="37"/>
-      <c r="F19" s="37"/>
-      <c r="G19" s="37"/>
-      <c r="H19" s="38"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
+      <c r="D19" s="29"/>
+      <c r="E19" s="29"/>
+      <c r="F19" s="29"/>
+      <c r="G19" s="29"/>
+      <c r="H19" s="30"/>
       <c r="I19"/>
       <c r="J19"/>
       <c r="K19"/>
@@ -2210,16 +2220,16 @@
       <c r="AQ26"/>
     </row>
     <row r="27" spans="1:43" s="2" customFormat="1" ht="18" x14ac:dyDescent="0.25">
-      <c r="A27" s="36" t="s">
+      <c r="A27" s="28" t="s">
         <v>20</v>
       </c>
-      <c r="B27" s="37"/>
-      <c r="C27" s="37"/>
-      <c r="D27" s="37"/>
-      <c r="E27" s="37"/>
-      <c r="F27" s="37"/>
-      <c r="G27" s="37"/>
-      <c r="H27" s="38"/>
+      <c r="B27" s="29"/>
+      <c r="C27" s="29"/>
+      <c r="D27" s="29"/>
+      <c r="E27" s="29"/>
+      <c r="F27" s="29"/>
+      <c r="G27" s="29"/>
+      <c r="H27" s="30"/>
       <c r="I27"/>
       <c r="J27"/>
       <c r="K27"/>
@@ -2672,6 +2682,11 @@
     <row r="81" customFormat="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="G1:H1"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="F3:H3"/>
     <mergeCell ref="A6:A7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A8:H8"/>
@@ -2679,11 +2694,6 @@
     <mergeCell ref="A27:H27"/>
     <mergeCell ref="B6:B7"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="G1:H1"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="F3:H3"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
@@ -2694,6 +2704,26 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a81de258-2782-43d6-9d1d-cd28d60619af">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="ed3c7b2c-ee95-4c62-b749-48a072e0fc6f" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101009F94F24C812C1443AF756F3262092C76" ma:contentTypeVersion="12" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="151ba19e32653bee0a5eee1707588175">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="a81de258-2782-43d6-9d1d-cd28d60619af" xmlns:ns3="ed3c7b2c-ee95-4c62-b749-48a072e0fc6f" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="177f0ace5463b349477f87f1b4642be3" ns2:_="" ns3:_="">
     <xsd:import namespace="a81de258-2782-43d6-9d1d-cd28d60619af"/>
@@ -2894,27 +2924,26 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76E9F743-2553-4538-B86E-9E9E949B7313}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a81de258-2782-43d6-9d1d-cd28d60619af"/>
+    <ds:schemaRef ds:uri="ed3c7b2c-ee95-4c62-b749-48a072e0fc6f"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="a81de258-2782-43d6-9d1d-cd28d60619af">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="ed3c7b2c-ee95-4c62-b749-48a072e0fc6f" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AE36CC0-C123-4309-B645-BEFA7CB5FE5A}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4E8AC1FA-2BD8-42E8-B266-319DE6BBF638}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -2931,23 +2960,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9AE36CC0-C123-4309-B645-BEFA7CB5FE5A}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76E9F743-2553-4538-B86E-9E9E949B7313}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="a81de258-2782-43d6-9d1d-cd28d60619af"/>
-    <ds:schemaRef ds:uri="ed3c7b2c-ee95-4c62-b749-48a072e0fc6f"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>